<commit_message>
update description statusAuthor 32a0be223d576a8d65272b9c5d8e84e510544189
</commit_message>
<xml_diff>
--- a/420-contenu-fhir---mise-à-jour-de-lévaluation/ig/StructureDefinition-tddui-careplan-projet-personnalise.xlsx
+++ b/420-contenu-fhir---mise-à-jour-de-lévaluation/ig/StructureDefinition-tddui-careplan-projet-personnalise.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-16T09:05:27+00:00</t>
+    <t>2026-02-23T08:45:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1012,7 +1012,7 @@
     <t>TDDUI Status Author</t>
   </si>
   <si>
-    <t>Extension permettant de représenter la profession du professionnel.</t>
+    <t>Extension permettant de représenter l'auteur du statut.</t>
   </si>
   <si>
     <t>statutProjetPersonnalise.auteur</t>

</xml_diff>